<commit_message>
Add Sai Shankar Sinha (25E51A66F1) and Sravani Gugulothu (23E51A05G0) to Mobile App Developer track
</commit_message>
<xml_diff>
--- a/backend/data/Student_Responses.xlsx
+++ b/backend/data/Student_Responses.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,12 +57,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>46250.77813372685</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -536,10 +536,9 @@
           <t>https://drive.google.com/open?id=1IVR89Sp7VWhBbmkqKhyw02mpVH1L1fXb</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>46250.77831935186</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -585,10 +584,9 @@
           <t>https://drive.google.com/open?id=15tZl1_iRpRzU1dsJ0OK7y40xOpr-q-ND</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>46250.79188813658</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -634,10 +632,9 @@
           <t>https://drive.google.com/open?id=1EdOn5d8SDlJub6T-iNtInJ7SQe1yILLo</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>46250.79446368056</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -683,10 +680,9 @@
           <t>https://drive.google.com/open?id=1rIumwAv6gH2HM-bcW8RYMpBo7eFOzyP-</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>46250.79970981481</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -732,10 +728,9 @@
           <t>https://drive.google.com/open?id=16TzPqcXqk4jUcjIyR-DIQjQdLaX7PqNY</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>46250.80266655092</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -781,10 +776,9 @@
           <t>https://drive.google.com/open?id=1E8K2mvr1JBXAiruKuEd_gZqf81LMtAJ_</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>46250.80278746528</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -830,10 +824,9 @@
           <t>https://drive.google.com/open?id=1BtSsd-TGMZy2tqhxvTnf6XWRHAajZYDd</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>46250.80292862269</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -879,10 +872,9 @@
           <t>https://drive.google.com/open?id=1nYc75IAxUyBfNlTa_ZdE4oN4l7089neB</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>46250.80974611111</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -928,10 +920,9 @@
           <t>https://drive.google.com/open?id=1lKqdstpwh6G5tHkrLJk5qk31Xrnba3UZ</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>46250.81495601852</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -984,7 +975,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>46250.81497548611</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -1037,7 +1028,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="3" t="n">
         <v>46250.83230452547</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1083,10 +1074,9 @@
           <t>https://drive.google.com/open?id=1eKGIkVhEvKLGya7NNCiqynm-jBmig_8W</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="3" t="n">
         <v>46250.85224311343</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1132,10 +1122,9 @@
           <t>https://drive.google.com/open?id=155ERIn5upkhNOKL1zr0YQsO_DrIMnJl0</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="3" t="n">
         <v>46250.85361491898</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1181,10 +1170,9 @@
           <t>https://drive.google.com/open?id=1LESHbBHoviTECng4AhZg9HL4wI8Y-njS</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="3" t="n">
         <v>46250.85384263889</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1237,7 +1225,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="3" t="n">
         <v>46250.85500270833</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1283,10 +1271,9 @@
           <t>https://drive.google.com/open?id=1LsSLITiBDsFEAAgAa_Wa2l0QskrxcucX</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="3" t="n">
         <v>46250.85993758102</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1332,10 +1319,9 @@
           <t>https://drive.google.com/open?id=1iumbm4WXjEZHjwAb5vOi_KROqJTTcmED</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="3" t="n">
         <v>46250.86195653935</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1381,10 +1367,9 @@
           <t>https://drive.google.com/open?id=1YZI3qZ0CKLrwHDN0VxN0yrpCgomWeeNg</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="3" t="n">
         <v>46250.86253388889</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1430,10 +1415,9 @@
           <t>https://drive.google.com/open?id=16-UH_OdVh0k6Mal9qH83y6QA03RrF8xb</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="3" t="n">
         <v>46250.86718664352</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1479,10 +1463,9 @@
           <t>https://drive.google.com/open?id=1WyBBiI7cDVnghyKvDT9YwH6-a-SKupqx</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="3" t="n">
         <v>46250.86771969908</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1528,10 +1511,9 @@
           <t>https://drive.google.com/open?id=1KB9A39MslylzvqPeDDkSilpaN2dy6N9_</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="3" t="n">
         <v>46250.86853123843</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1582,7 +1564,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="3" t="n">
         <v>46250.86948836806</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1628,10 +1610,9 @@
           <t>https://drive.google.com/open?id=1Y8x5TlDv5bQ2VZnjbM-ap5U67aFvZj-v</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="3" t="n">
         <v>46250.87093619213</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1677,10 +1658,9 @@
           <t>https://drive.google.com/open?id=15zqiVAom_opNigxGijszlfNAKojWKRTI</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="3" t="n">
         <v>46250.87211105324</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1726,10 +1706,9 @@
           <t>https://drive.google.com/open?id=1BAn46HarZcLSBRxlF9cW4VR9sJ7tphTl</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="3" t="n">
         <v>46250.87406452547</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1775,10 +1754,9 @@
           <t>https://drive.google.com/open?id=14OI31JfoQeDAw3C7gh4s7iotsjx2ZKky</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="3" t="n">
         <v>46250.87408222222</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1824,10 +1802,9 @@
           <t>https://drive.google.com/open?id=14E9lJuF6I-JlB7rL69TSXu0kPuGsYsk-</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="3" t="n">
         <v>46250.87415837963</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1875,10 +1852,9 @@
           <t>https://drive.google.com/open?id=1NRJmqdpZ-0FVuEYW9ZVya3n_hUHHjMwx</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="3" t="n">
         <v>46250.87494894676</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1924,10 +1900,9 @@
           <t>https://drive.google.com/open?id=16npsQWeOtkifhGAdHgr0U5scMTu-AN42</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="3" t="n">
         <v>46250.87511645833</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1973,10 +1948,9 @@
           <t>https://drive.google.com/open?id=1bpKXnpIxdJi2KlQYIvP2R_-4LZIeSZVe</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="3" t="n">
         <v>46250.87566009259</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -2022,10 +1996,9 @@
           <t>https://drive.google.com/open?id=1jKgG_MR8lB6jbAauaGU-EWjovjB2FdEy</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="3" t="n">
         <v>46250.87597190972</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -2071,10 +2044,9 @@
           <t>https://drive.google.com/open?id=12longhwVIm4T_1kQiLxe7YrJgrEu68ZP</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="3" t="n">
         <v>46250.87698282408</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -2120,10 +2092,9 @@
           <t>https://drive.google.com/open?id=1TC5fBWEJ6iMrPh28L5uFgsp3dGlCelGC</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="3" t="n">
         <v>46250.87800190972</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -2169,10 +2140,9 @@
           <t>https://drive.google.com/open?id=1g3WgjLvP9vB_4ozAajFbuo3Cu1OHd7y0</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="3" t="n">
         <v>46250.87815363426</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -2218,10 +2188,9 @@
           <t>https://drive.google.com/open?id=19np5eQs__h0Mmwg8Bhj8WdM4ctdbUHvU</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="3" t="n">
         <v>46250.87820583333</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -2267,10 +2236,9 @@
           <t>https://drive.google.com/open?id=1YHsJIE8Bjdmp-mhKGzAQqhvzdhL2nxum</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="3" t="n">
         <v>46250.87959746527</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -2316,10 +2284,9 @@
           <t>https://drive.google.com/open?id=1WE0ySsgcGTcuHzEsW6zqfEG1fcg9kpvO</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="3" t="n">
         <v>46250.87995774305</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -2365,10 +2332,9 @@
           <t>https://drive.google.com/open?id=1gxh356_xEDqtpfrIOSDHwEOZq3BGZMpN</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="3" t="n">
         <v>46250.88157581018</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -2414,10 +2380,9 @@
           <t>https://drive.google.com/open?id=1ZtNPzM5pScpB33jFGPYNFFpzAggImaB7</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="3" t="n">
         <v>46250.88984047453</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -2463,10 +2428,9 @@
           <t>https://drive.google.com/open?id=1SGpA3dkuG6KcyACC8xz389lMLIMlAX7B</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="3" t="n">
         <v>46250.89788890046</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -2512,10 +2476,9 @@
           <t>https://drive.google.com/open?id=1db2vp70dZBeHIG-egxpRJG833aUMv8Gn</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="3" t="n">
         <v>46250.90032488426</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -2568,7 +2531,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="3" t="n">
         <v>46250.92399141203</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -2614,10 +2577,9 @@
           <t>https://drive.google.com/open?id=1fWBqJ2PBVAVDJdSO6oUMyQjdvTKUTvEb</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="3" t="n">
         <v>46250.92569491898</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -2663,10 +2625,9 @@
           <t>https://drive.google.com/open?id=1yTc3O6vdSLgm4W7EU4_yfEh2pIzcbf1c</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="3" t="n">
         <v>46250.9534227662</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -2712,10 +2673,9 @@
           <t>https://drive.google.com/open?id=1u7t0mMDVe1yBx1Gr6ZjYELgeqxnXjjUG</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="3" t="n">
         <v>46250.95407225694</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -2761,10 +2721,9 @@
           <t>https://drive.google.com/open?id=1jPpRygC8c3voRUb0xf0D11CTa0iH7IWb</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="3" t="n">
         <v>46250.96036038194</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -2810,10 +2769,9 @@
           <t>https://drive.google.com/open?id=1BmVQvGew4FwRIfFMRJgxc8FdR2ECBbYg</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="3" t="n">
         <v>46250.96319504629</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -2859,10 +2817,9 @@
           <t>https://drive.google.com/open?id=1xgmkVDVxUTpZanZtfRQ16Biriz0dsqwa</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="3" t="n">
         <v>46250.97590630787</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -2908,10 +2865,9 @@
           <t>https://drive.google.com/open?id=1KMHd8W7lICf8uXZbS1xreqVZuHPtBupd</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="3" t="n">
         <v>46251.00046760416</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -2957,10 +2913,9 @@
           <t>https://drive.google.com/open?id=1WqohCJuEwYzLBBEgQKQJySfSLw_eq6J0</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="3" t="n">
         <v>46251.24788288194</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -3006,10 +2961,9 @@
           <t>https://drive.google.com/open?id=1kHlx8k3yRRko0Uxp5JlHGc_72o1yjfmF</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="3" t="n">
         <v>46251.38022956019</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -3062,7 +3016,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="3" t="n">
         <v>46251.38457657408</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -3070,7 +3024,6 @@
           <t>Gm Aravind</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>gmarav005@gmail.com</t>
@@ -3111,7 +3064,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="3" t="n">
         <v>46251.38572273148</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -3157,10 +3110,9 @@
           <t>https://drive.google.com/open?id=1ViKz5dUWFSkA7Gt75-IAR_XQOXiKhak2</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="3" t="n">
         <v>46251.38650766204</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -3206,10 +3158,9 @@
           <t>https://drive.google.com/open?id=1xlZKrrfkoMHWJnEdhszY-8PiHvHHs4E4</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="3" t="n">
         <v>46251.38837877315</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -3255,10 +3206,9 @@
           <t>https://drive.google.com/open?id=1CdZ3AKbN_GrG4H4dmzY-9JK0LeEur0sc</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="3" t="n">
         <v>46251.39116122685</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -3304,10 +3254,9 @@
           <t>https://drive.google.com/open?id=1-_FqiQd9vJn1KtwUZ9AMaDR7hUIQJUe0</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="3" t="n">
         <v>46251.39235314815</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -3353,10 +3302,9 @@
           <t>https://drive.google.com/open?id=1rVqZVREnqThBtn4kaAeJyUXFUKJWVMnE</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="3" t="n">
         <v>46251.39488421296</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -3402,10 +3350,9 @@
           <t>https://drive.google.com/open?id=1wfSkqmCfs-nd8fOpDSDKaTrw7-z8Uczo</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="3" t="n">
         <v>46251.39605935185</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -3451,10 +3398,9 @@
           <t>https://drive.google.com/open?id=1SI2zm1dwfr-IFk-67V-AcKSmEM-xkGCs</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="3" t="n">
         <v>46251.40607896991</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -3500,10 +3446,9 @@
           <t>https://drive.google.com/open?id=11gjqpiyONeKhCSSWjS1rPqV3TFiMZ0kK</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="3" t="n">
         <v>46251.41115348379</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -3549,10 +3494,9 @@
           <t>https://drive.google.com/open?id=1yaadLJ5zgOYK-WeSxatDHQLKepkhSud9</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="3" t="n">
         <v>46251.42504689815</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -3598,10 +3542,9 @@
           <t>https://drive.google.com/open?id=1P0CZWJWhBe_wPUVHJ7XOssCo4CJhKnRM</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="3" t="n">
         <v>46251.42519075231</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -3652,7 +3595,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="3" t="n">
         <v>46251.45734157407</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -3698,10 +3641,9 @@
           <t>https://drive.google.com/open?id=1l8pVNWacQ40UW7NJjieXtBa-C7p2dwos</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="3" t="n">
         <v>46251.50740381944</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -3747,10 +3689,9 @@
           <t>https://drive.google.com/open?id=1GcaUFfZiAYz5QYcgLmccbaBzv5wHnkFo</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="3" t="n">
         <v>46251.55135984954</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -3796,10 +3737,9 @@
           <t>https://drive.google.com/open?id=1Oli5KQ8KL9rfLEKMU7k4l8XNRBk1Xu3W</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="3" t="n">
         <v>46251.79081414352</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -3845,10 +3785,9 @@
           <t>https://drive.google.com/open?id=11w9S-pzxLfaH_TnOxI0HqFRn3X-0tUjG</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="3" t="n">
         <v>46251.87708452546</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -3894,10 +3833,9 @@
           <t>https://drive.google.com/open?id=1mIiugddHZjPQKdiCAS9uIR9TN13WBWLw</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="3" t="n">
         <v>46251.90245274305</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -3943,10 +3881,9 @@
           <t>https://drive.google.com/open?id=1-bkk5CjN4FKvfI35NNMA0Eg-6dc0F1uT</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="3" t="n">
         <v>46251.91770545139</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -3992,10 +3929,9 @@
           <t>https://drive.google.com/open?id=1lmrEQ67TpM_rrrv--qRIYiazVO3xyJFr</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="3" t="n">
         <v>46252.40242706019</v>
       </c>
       <c r="B73" t="inlineStr">
@@ -4041,10 +3977,9 @@
           <t>https://drive.google.com/open?id=1AWvt7OihNfhkIk2QRr2xYHIzdzXlRr4P</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="3" t="n">
         <v>46252.41530847222</v>
       </c>
       <c r="B74" t="inlineStr">
@@ -4090,10 +4025,9 @@
           <t>https://drive.google.com/open?id=1GoYn1VjlV2Hw2SdZkzxNh3dT9v_ci6k1</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="3" t="n">
         <v>46252.41630350694</v>
       </c>
       <c r="B75" t="inlineStr">
@@ -4139,10 +4073,9 @@
           <t>https://drive.google.com/open?id=1lvjSUiCV-zB632yLDxrpbVnXUlJF7mmT</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="3" t="n">
         <v>46252.46472571759</v>
       </c>
       <c r="B76" t="inlineStr">
@@ -4188,10 +4121,9 @@
           <t>https://drive.google.com/open?id=14Z45g9mwfXiIO2srsYABnFnfLuYz61Xz</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="3" t="n">
         <v>46253.82424209491</v>
       </c>
       <c r="B77" t="inlineStr">
@@ -4244,7 +4176,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="3" t="n">
         <v>46253.85308646991</v>
       </c>
       <c r="B78" t="inlineStr">
@@ -4297,7 +4229,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="3" t="n">
         <v>46253.89656041667</v>
       </c>
       <c r="B79" t="inlineStr">
@@ -4350,7 +4282,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="3" t="n">
         <v>46254.94776509259</v>
       </c>
       <c r="B80" t="inlineStr">
@@ -4396,10 +4328,9 @@
           <t>https://drive.google.com/open?id=1xURMC_EP1hiA0OOlDqMkyRMWoR2JD6vc</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="3" t="n">
         <v>46267.35141709491</v>
       </c>
       <c r="B81" t="inlineStr">
@@ -4445,10 +4376,9 @@
           <t>https://drive.google.com/open?id=1uHuv5xCr8HD1549LWhzQuZ7F_TMvwDtM</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="3" t="n">
         <v>46267.41529385417</v>
       </c>
       <c r="B82" t="inlineStr">
@@ -4494,10 +4424,9 @@
           <t>https://drive.google.com/open?id=1kLddUqGybcQ9v5gFu2aawkROvrbuDbpf</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="3" t="n">
         <v>46267.46011768519</v>
       </c>
       <c r="B83" t="inlineStr">
@@ -4543,10 +4472,9 @@
           <t>https://drive.google.com/open?id=1zeq1dZY4EZC0UTslB04e55nrV8XbvxpJ</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="3" t="n">
         <v>46267.48658503472</v>
       </c>
       <c r="B84" t="inlineStr">
@@ -4592,10 +4520,9 @@
           <t>https://drive.google.com/open?id=1tmB5IUGNw_YwWO77BJTi4X2s4_lw4Tma</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="3" t="n">
         <v>46267.48737980324</v>
       </c>
       <c r="B85" t="inlineStr">
@@ -4641,10 +4568,9 @@
           <t>https://drive.google.com/open?id=1xR7RHFRAQTwrebbFHQQObbrFcJEJLK5f</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="3" t="n">
         <v>46267.79814045139</v>
       </c>
       <c r="B86" t="inlineStr">
@@ -4690,10 +4616,9 @@
           <t>https://drive.google.com/open?id=1_5P7Tnj-P8LbZDpDBWE1UtHXyWvPbkxE</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="3" t="n">
         <v>46268.09300221065</v>
       </c>
       <c r="B87" t="inlineStr">
@@ -4739,7 +4664,56 @@
           <t>https://drive.google.com/open?id=13KakKIzib8bVbRKtU4IfXsGbQEWfNCMr</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sai Shankar Sinha</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>25E51A66F1</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Cse in aiml</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Mobile App Developer Intern</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Sravani Gugulothu</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23E51A05G0</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Mobile App Developer Intern</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>